<commit_message>
ONESHOT m5: slutrapport — v2 klar, regression gron, print_preview.pdf
10 flikar trogen-verifierade. Oversikt 18->1 sida, Kassaflode 10->2,
Grafer ny, 6 produktionsbuggar i iter9 dokumenterade och fixade i v2
(F-1 locale-TEXT, F-3 #NAME?, F-4 stale refs, F-5 dod INFASNING,
F-6 trasig print, Dokumentation-klippning). Baslinje exakt:
11 631 221,72 / 7,6452 % / +1,35 pp. Noll formelfel.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/oneshot/Investeringskalkyl_v2.xlsx
+++ b/build/oneshot/Investeringskalkyl_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaki\Documents\GitHub\investeringskalkyl\build\oneshot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4E9C4CD-F60B-42D7-8063-58FB8E2C6E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53774B03-CC2C-4953-9660-CBF61CF32018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="345" yWindow="345" windowWidth="28800" windowHeight="16065" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3098,7 +3098,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-733A-4FAB-A948-4C7F32C921FE}"/>
+              <c16:uniqueId val="{00000000-ADD1-46F7-9AEF-1AE39D97D7A7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3349,7 +3349,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B7B7-4FE9-A896-E274BA52FBD9}"/>
+              <c16:uniqueId val="{00000000-302C-4D76-8516-FBF4F1C370A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3511,7 +3511,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B7B7-4FE9-A896-E274BA52FBD9}"/>
+              <c16:uniqueId val="{00000001-302C-4D76-8516-FBF4F1C370A4}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3672,7 +3672,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-CFAC-4A2C-942F-39E826F4D054}"/>
+              <c16:uniqueId val="{00000000-33B2-432D-8F02-AB7C983860A7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -15797,66 +15797,21 @@
         <f>IF(OR(Indata!$K$26="",M$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*M$16)</f>
         <v>13181563.602194397</v>
       </c>
-      <c r="N30" s="20">
-        <f>IF(OR(Indata!$K$26="",N$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*N$16)</f>
-        <v>0</v>
-      </c>
-      <c r="O30" s="20">
-        <f>IF(OR(Indata!$K$26="",O$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*O$16)</f>
-        <v>0</v>
-      </c>
-      <c r="P30" s="20">
-        <f>IF(OR(Indata!$K$26="",P$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*P$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Q30" s="20">
-        <f>IF(OR(Indata!$K$26="",Q$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*Q$16)</f>
-        <v>0</v>
-      </c>
-      <c r="R30" s="20">
-        <f>IF(OR(Indata!$K$26="",R$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*R$16)</f>
-        <v>0</v>
-      </c>
-      <c r="S30" s="20">
-        <f>IF(OR(Indata!$K$26="",S$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*S$16)</f>
-        <v>0</v>
-      </c>
-      <c r="T30" s="20">
-        <f>IF(OR(Indata!$K$26="",T$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*T$16)</f>
-        <v>0</v>
-      </c>
-      <c r="U30" s="20">
-        <f>IF(OR(Indata!$K$26="",U$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*U$16)</f>
-        <v>0</v>
-      </c>
-      <c r="V30" s="20">
-        <f>IF(OR(Indata!$K$26="",V$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*V$16)</f>
-        <v>0</v>
-      </c>
-      <c r="W30" s="20">
-        <f>IF(OR(Indata!$K$26="",W$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*W$16)</f>
-        <v>0</v>
-      </c>
-      <c r="X30" s="20">
-        <f>IF(OR(Indata!$K$26="",X$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*X$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Y30" s="20">
-        <f>IF(OR(Indata!$K$26="",Y$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*Y$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Z30" s="20">
-        <f>IF(OR(Indata!$K$26="",Z$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*Z$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AA30" s="20">
-        <f>IF(OR(Indata!$K$26="",AA$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*AA$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AB30" s="20">
-        <f>IF(OR(Indata!$K$26="",AB$29&lt;Indata!$K$26),0,(Indata!$R$26/Indata!$R$31)*AB$16)</f>
-        <v>0</v>
-      </c>
+      <c r="N30" s="20"/>
+      <c r="O30" s="20"/>
+      <c r="P30" s="20"/>
+      <c r="Q30" s="20"/>
+      <c r="R30" s="20"/>
+      <c r="S30" s="20"/>
+      <c r="T30" s="20"/>
+      <c r="U30" s="20"/>
+      <c r="V30" s="20"/>
+      <c r="W30" s="20"/>
+      <c r="X30" s="20"/>
+      <c r="Y30" s="20"/>
+      <c r="Z30" s="20"/>
+      <c r="AA30" s="20"/>
+      <c r="AB30" s="20"/>
     </row>
     <row r="31" spans="1:28" ht="15" customHeight="1">
       <c r="A31" s="19"/>
@@ -15905,66 +15860,21 @@
         <f>IF(OR(Indata!$K$27="",M$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*M$16)</f>
         <v>0</v>
       </c>
-      <c r="N31" s="20">
-        <f>IF(OR(Indata!$K$27="",N$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*N$16)</f>
-        <v>0</v>
-      </c>
-      <c r="O31" s="20">
-        <f>IF(OR(Indata!$K$27="",O$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*O$16)</f>
-        <v>0</v>
-      </c>
-      <c r="P31" s="20">
-        <f>IF(OR(Indata!$K$27="",P$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*P$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Q31" s="20">
-        <f>IF(OR(Indata!$K$27="",Q$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*Q$16)</f>
-        <v>0</v>
-      </c>
-      <c r="R31" s="20">
-        <f>IF(OR(Indata!$K$27="",R$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*R$16)</f>
-        <v>0</v>
-      </c>
-      <c r="S31" s="20">
-        <f>IF(OR(Indata!$K$27="",S$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*S$16)</f>
-        <v>0</v>
-      </c>
-      <c r="T31" s="20">
-        <f>IF(OR(Indata!$K$27="",T$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*T$16)</f>
-        <v>0</v>
-      </c>
-      <c r="U31" s="20">
-        <f>IF(OR(Indata!$K$27="",U$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*U$16)</f>
-        <v>0</v>
-      </c>
-      <c r="V31" s="20">
-        <f>IF(OR(Indata!$K$27="",V$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*V$16)</f>
-        <v>0</v>
-      </c>
-      <c r="W31" s="20">
-        <f>IF(OR(Indata!$K$27="",W$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*W$16)</f>
-        <v>0</v>
-      </c>
-      <c r="X31" s="20">
-        <f>IF(OR(Indata!$K$27="",X$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*X$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Y31" s="20">
-        <f>IF(OR(Indata!$K$27="",Y$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*Y$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Z31" s="20">
-        <f>IF(OR(Indata!$K$27="",Z$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*Z$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AA31" s="20">
-        <f>IF(OR(Indata!$K$27="",AA$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*AA$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AB31" s="20">
-        <f>IF(OR(Indata!$K$27="",AB$29&lt;Indata!$K$27),0,(Indata!$R$27/Indata!$R$31)*AB$16)</f>
-        <v>0</v>
-      </c>
+      <c r="N31" s="20"/>
+      <c r="O31" s="20"/>
+      <c r="P31" s="20"/>
+      <c r="Q31" s="20"/>
+      <c r="R31" s="20"/>
+      <c r="S31" s="20"/>
+      <c r="T31" s="20"/>
+      <c r="U31" s="20"/>
+      <c r="V31" s="20"/>
+      <c r="W31" s="20"/>
+      <c r="X31" s="20"/>
+      <c r="Y31" s="20"/>
+      <c r="Z31" s="20"/>
+      <c r="AA31" s="20"/>
+      <c r="AB31" s="20"/>
     </row>
     <row r="32" spans="1:28" ht="21.75" customHeight="1">
       <c r="A32" s="19"/>
@@ -16013,66 +15923,21 @@
         <f>IF(OR(Indata!$K$28="",M$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*M$16)</f>
         <v>0</v>
       </c>
-      <c r="N32" s="20">
-        <f>IF(OR(Indata!$K$28="",N$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*N$16)</f>
-        <v>0</v>
-      </c>
-      <c r="O32" s="20">
-        <f>IF(OR(Indata!$K$28="",O$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*O$16)</f>
-        <v>0</v>
-      </c>
-      <c r="P32" s="20">
-        <f>IF(OR(Indata!$K$28="",P$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*P$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Q32" s="20">
-        <f>IF(OR(Indata!$K$28="",Q$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*Q$16)</f>
-        <v>0</v>
-      </c>
-      <c r="R32" s="20">
-        <f>IF(OR(Indata!$K$28="",R$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*R$16)</f>
-        <v>0</v>
-      </c>
-      <c r="S32" s="20">
-        <f>IF(OR(Indata!$K$28="",S$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*S$16)</f>
-        <v>0</v>
-      </c>
-      <c r="T32" s="20">
-        <f>IF(OR(Indata!$K$28="",T$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*T$16)</f>
-        <v>0</v>
-      </c>
-      <c r="U32" s="20">
-        <f>IF(OR(Indata!$K$28="",U$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*U$16)</f>
-        <v>0</v>
-      </c>
-      <c r="V32" s="20">
-        <f>IF(OR(Indata!$K$28="",V$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*V$16)</f>
-        <v>0</v>
-      </c>
-      <c r="W32" s="20">
-        <f>IF(OR(Indata!$K$28="",W$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*W$16)</f>
-        <v>0</v>
-      </c>
-      <c r="X32" s="20">
-        <f>IF(OR(Indata!$K$28="",X$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*X$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Y32" s="20">
-        <f>IF(OR(Indata!$K$28="",Y$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*Y$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Z32" s="20">
-        <f>IF(OR(Indata!$K$28="",Z$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*Z$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AA32" s="20">
-        <f>IF(OR(Indata!$K$28="",AA$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*AA$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AB32" s="20">
-        <f>IF(OR(Indata!$K$28="",AB$29&lt;Indata!$K$28),0,(Indata!$R$28/Indata!$R$31)*AB$16)</f>
-        <v>0</v>
-      </c>
+      <c r="N32" s="20"/>
+      <c r="O32" s="20"/>
+      <c r="P32" s="20"/>
+      <c r="Q32" s="20"/>
+      <c r="R32" s="20"/>
+      <c r="S32" s="20"/>
+      <c r="T32" s="20"/>
+      <c r="U32" s="20"/>
+      <c r="V32" s="20"/>
+      <c r="W32" s="20"/>
+      <c r="X32" s="20"/>
+      <c r="Y32" s="20"/>
+      <c r="Z32" s="20"/>
+      <c r="AA32" s="20"/>
+      <c r="AB32" s="20"/>
     </row>
     <row r="33" spans="1:28" ht="15" customHeight="1">
       <c r="A33" s="19"/>
@@ -16121,66 +15986,21 @@
         <f>IF(OR(Indata!$K$29="",M$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*M$16)</f>
         <v>0</v>
       </c>
-      <c r="N33" s="20">
-        <f>IF(OR(Indata!$K$29="",N$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*N$16)</f>
-        <v>0</v>
-      </c>
-      <c r="O33" s="20">
-        <f>IF(OR(Indata!$K$29="",O$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*O$16)</f>
-        <v>0</v>
-      </c>
-      <c r="P33" s="20">
-        <f>IF(OR(Indata!$K$29="",P$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*P$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Q33" s="20">
-        <f>IF(OR(Indata!$K$29="",Q$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*Q$16)</f>
-        <v>0</v>
-      </c>
-      <c r="R33" s="20">
-        <f>IF(OR(Indata!$K$29="",R$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*R$16)</f>
-        <v>0</v>
-      </c>
-      <c r="S33" s="20">
-        <f>IF(OR(Indata!$K$29="",S$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*S$16)</f>
-        <v>0</v>
-      </c>
-      <c r="T33" s="20">
-        <f>IF(OR(Indata!$K$29="",T$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*T$16)</f>
-        <v>0</v>
-      </c>
-      <c r="U33" s="20">
-        <f>IF(OR(Indata!$K$29="",U$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*U$16)</f>
-        <v>0</v>
-      </c>
-      <c r="V33" s="20">
-        <f>IF(OR(Indata!$K$29="",V$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*V$16)</f>
-        <v>0</v>
-      </c>
-      <c r="W33" s="20">
-        <f>IF(OR(Indata!$K$29="",W$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*W$16)</f>
-        <v>0</v>
-      </c>
-      <c r="X33" s="20">
-        <f>IF(OR(Indata!$K$29="",X$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*X$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Y33" s="20">
-        <f>IF(OR(Indata!$K$29="",Y$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*Y$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Z33" s="20">
-        <f>IF(OR(Indata!$K$29="",Z$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*Z$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AA33" s="20">
-        <f>IF(OR(Indata!$K$29="",AA$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*AA$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AB33" s="20">
-        <f>IF(OR(Indata!$K$29="",AB$29&lt;Indata!$K$29),0,(Indata!$R$29/Indata!$R$31)*AB$16)</f>
-        <v>0</v>
-      </c>
+      <c r="N33" s="20"/>
+      <c r="O33" s="20"/>
+      <c r="P33" s="20"/>
+      <c r="Q33" s="20"/>
+      <c r="R33" s="20"/>
+      <c r="S33" s="20"/>
+      <c r="T33" s="20"/>
+      <c r="U33" s="20"/>
+      <c r="V33" s="20"/>
+      <c r="W33" s="20"/>
+      <c r="X33" s="20"/>
+      <c r="Y33" s="20"/>
+      <c r="Z33" s="20"/>
+      <c r="AA33" s="20"/>
+      <c r="AB33" s="20"/>
     </row>
     <row r="34" spans="1:28" ht="15" customHeight="1">
       <c r="A34" s="19"/>
@@ -16229,66 +16049,21 @@
         <f>IF(OR(Indata!$K$30="",M$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*M$16)</f>
         <v>0</v>
       </c>
-      <c r="N34" s="20">
-        <f>IF(OR(Indata!$K$30="",N$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*N$16)</f>
-        <v>0</v>
-      </c>
-      <c r="O34" s="20">
-        <f>IF(OR(Indata!$K$30="",O$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*O$16)</f>
-        <v>0</v>
-      </c>
-      <c r="P34" s="20">
-        <f>IF(OR(Indata!$K$30="",P$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*P$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Q34" s="20">
-        <f>IF(OR(Indata!$K$30="",Q$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*Q$16)</f>
-        <v>0</v>
-      </c>
-      <c r="R34" s="20">
-        <f>IF(OR(Indata!$K$30="",R$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*R$16)</f>
-        <v>0</v>
-      </c>
-      <c r="S34" s="20">
-        <f>IF(OR(Indata!$K$30="",S$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*S$16)</f>
-        <v>0</v>
-      </c>
-      <c r="T34" s="20">
-        <f>IF(OR(Indata!$K$30="",T$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*T$16)</f>
-        <v>0</v>
-      </c>
-      <c r="U34" s="20">
-        <f>IF(OR(Indata!$K$30="",U$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*U$16)</f>
-        <v>0</v>
-      </c>
-      <c r="V34" s="20">
-        <f>IF(OR(Indata!$K$30="",V$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*V$16)</f>
-        <v>0</v>
-      </c>
-      <c r="W34" s="20">
-        <f>IF(OR(Indata!$K$30="",W$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*W$16)</f>
-        <v>0</v>
-      </c>
-      <c r="X34" s="20">
-        <f>IF(OR(Indata!$K$30="",X$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*X$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Y34" s="20">
-        <f>IF(OR(Indata!$K$30="",Y$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*Y$16)</f>
-        <v>0</v>
-      </c>
-      <c r="Z34" s="20">
-        <f>IF(OR(Indata!$K$30="",Z$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*Z$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AA34" s="20">
-        <f>IF(OR(Indata!$K$30="",AA$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*AA$16)</f>
-        <v>0</v>
-      </c>
-      <c r="AB34" s="20">
-        <f>IF(OR(Indata!$K$30="",AB$29&lt;Indata!$K$30),0,(Indata!$R$30/Indata!$R$31)*AB$16)</f>
-        <v>0</v>
-      </c>
+      <c r="N34" s="20"/>
+      <c r="O34" s="20"/>
+      <c r="P34" s="20"/>
+      <c r="Q34" s="20"/>
+      <c r="R34" s="20"/>
+      <c r="S34" s="20"/>
+      <c r="T34" s="20"/>
+      <c r="U34" s="20"/>
+      <c r="V34" s="20"/>
+      <c r="W34" s="20"/>
+      <c r="X34" s="20"/>
+      <c r="Y34" s="20"/>
+      <c r="Z34" s="20"/>
+      <c r="AA34" s="20"/>
+      <c r="AB34" s="20"/>
     </row>
     <row r="35" spans="1:28" ht="15" customHeight="1">
       <c r="A35" s="19"/>
@@ -16359,7 +16134,7 @@
       </c>
       <c r="C36" s="20"/>
       <c r="D36" s="89">
-        <f t="shared" ref="D36:AB36" si="2">IFERROR(D35/D16,0)</f>
+        <f t="shared" ref="D36:M36" si="2">IFERROR(D35/D16,0)</f>
         <v>1</v>
       </c>
       <c r="E36" s="89">
@@ -16398,66 +16173,21 @@
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="N36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="O36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="P36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="R36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="S36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="T36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="U36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="V36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="W36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="X36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Y36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Z36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AA36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AB36" s="20">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="N36" s="20"/>
+      <c r="O36" s="20"/>
+      <c r="P36" s="20"/>
+      <c r="Q36" s="20"/>
+      <c r="R36" s="20"/>
+      <c r="S36" s="20"/>
+      <c r="T36" s="20"/>
+      <c r="U36" s="20"/>
+      <c r="V36" s="20"/>
+      <c r="W36" s="20"/>
+      <c r="X36" s="20"/>
+      <c r="Y36" s="20"/>
+      <c r="Z36" s="20"/>
+      <c r="AA36" s="20"/>
+      <c r="AB36" s="20"/>
     </row>
     <row r="37" spans="1:28" ht="15" customHeight="1">
       <c r="A37" s="19"/>

</xml_diff>

<commit_message>
Nav-knapparna klickbara: hyperlänk på bilderna via XML-patch
Cell-hyperlänkarna bakom knapp-PNG:erna nås aldrig med mus — bilden fångar
klicket, och på skyddade blad är bildobjekt utan egen länk döda. Ny
patch_nav_hyperlinks i post_save: a:hlinkClick först i cNvPr + hyperlink-
relationship (Target="#'Flik'!A1" TargetMode="External") per drawing.
100 länkar (10 knappar x 10 flikar), aktiv flik länkar till egen A1.

Läxor: openpyxl skriver drawing-XML med default-ns UTAN xdr:-prefix
(Excel-omsparning prefixar) — mönstren matchar båda formerna; insatt
element måste deklarera xmlns:a/xmlns:r inline, annars reparerar Excel
tyst bort alltihop vid recalc.

Verifierat: XML 100/100 efter recalc, COM Hyperlink.Follow 10/10 från
Översikt + från skyddat Försättsblad. Regression grön.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/build/oneshot/Investeringskalkyl_v2.xlsx
+++ b/build/oneshot/Investeringskalkyl_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaki\Documents\GitHub\investeringskalkyl\build\oneshot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F5E5AF6-260E-4CEF-9A2E-AEFDC472A58C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A1DA65-7EBD-4967-85BB-6DE2CABA4478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9615" yWindow="1875" windowWidth="28785" windowHeight="16065" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Översikt" sheetId="1" r:id="rId1"/>
@@ -3213,7 +3213,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E1BA-4AC6-8C67-057259410037}"/>
+              <c16:uniqueId val="{00000000-BA3E-44C0-A48A-A8A7229A56CD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3464,7 +3464,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-96BF-4404-8F02-4336DFA6D3D3}"/>
+              <c16:uniqueId val="{00000000-EE40-445F-8553-8368271BCCDF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3626,7 +3626,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-96BF-4404-8F02-4336DFA6D3D3}"/>
+              <c16:uniqueId val="{00000001-EE40-445F-8553-8368271BCCDF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3787,7 +3787,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-177F-4CB4-9A25-CB72A8E74FC3}"/>
+              <c16:uniqueId val="{00000000-92EF-48FF-A3CE-371148E22CAD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3863,6 +3863,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
@@ -3872,7 +3873,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3896,6 +3897,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
@@ -3905,7 +3907,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3929,6 +3931,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
@@ -3938,7 +3941,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3962,6 +3965,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
@@ -3971,7 +3975,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -3995,6 +3999,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000006000000}"/>
@@ -4004,7 +4009,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4028,6 +4033,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
@@ -4037,7 +4043,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4061,6 +4067,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
@@ -4070,7 +4077,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4094,6 +4101,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
@@ -4103,7 +4111,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4127,6 +4135,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000A000000}"/>
@@ -4136,7 +4145,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4160,6 +4169,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000B000000}"/>
@@ -4169,7 +4179,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4198,6 +4208,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-000002000000}"/>
@@ -4207,7 +4218,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4231,6 +4242,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-000003000000}"/>
@@ -4240,7 +4252,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4264,6 +4276,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-000004000000}"/>
@@ -4273,7 +4286,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4297,6 +4310,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-000005000000}"/>
@@ -4306,7 +4320,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4330,6 +4344,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-000006000000}"/>
@@ -4339,7 +4354,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4363,6 +4378,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-000007000000}"/>
@@ -4372,7 +4388,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4396,6 +4412,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-000008000000}"/>
@@ -4405,7 +4422,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4429,6 +4446,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-000009000000}"/>
@@ -4438,7 +4456,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4462,6 +4480,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-00000A000000}"/>
@@ -4471,7 +4490,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4495,6 +4514,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0900-00000B000000}"/>
@@ -4504,7 +4524,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4533,6 +4553,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
@@ -4542,7 +4563,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4566,6 +4587,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
@@ -4575,7 +4597,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4599,6 +4621,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000004000000}"/>
@@ -4608,7 +4631,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4632,6 +4655,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000005000000}"/>
@@ -4641,7 +4665,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4665,6 +4689,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000006000000}"/>
@@ -4674,7 +4699,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4698,6 +4723,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000007000000}"/>
@@ -4707,7 +4733,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4731,6 +4757,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000008000000}"/>
@@ -4740,7 +4767,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4764,6 +4791,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000009000000}"/>
@@ -4773,7 +4801,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4797,6 +4825,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-00000A000000}"/>
@@ -4806,7 +4835,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4830,6 +4859,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-00000B000000}"/>
@@ -4839,7 +4869,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4868,6 +4898,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
@@ -4877,7 +4908,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4901,6 +4932,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000003000000}"/>
@@ -4910,7 +4942,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4934,6 +4966,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000004000000}"/>
@@ -4943,7 +4976,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -4967,6 +5000,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000005000000}"/>
@@ -4976,7 +5010,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5000,6 +5034,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000006000000}"/>
@@ -5009,7 +5044,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5033,6 +5068,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000007000000}"/>
@@ -5042,7 +5078,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5066,6 +5102,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000008000000}"/>
@@ -5075,7 +5112,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5099,6 +5136,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000009000000}"/>
@@ -5108,7 +5146,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5132,6 +5170,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-00000A000000}"/>
@@ -5141,7 +5180,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5165,6 +5204,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-00000B000000}"/>
@@ -5174,7 +5214,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5203,6 +5243,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000002000000}"/>
@@ -5212,7 +5253,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5236,6 +5277,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000003000000}"/>
@@ -5245,7 +5287,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5269,6 +5311,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000004000000}"/>
@@ -5278,7 +5321,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5302,6 +5345,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000005000000}"/>
@@ -5311,7 +5355,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5335,6 +5379,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000006000000}"/>
@@ -5344,7 +5389,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5368,6 +5413,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000007000000}"/>
@@ -5377,7 +5423,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5401,6 +5447,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000008000000}"/>
@@ -5410,7 +5457,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5434,6 +5481,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000009000000}"/>
@@ -5443,7 +5491,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5467,6 +5515,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000A000000}"/>
@@ -5476,7 +5525,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5500,6 +5549,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000B000000}"/>
@@ -5509,7 +5559,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5538,6 +5588,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000002000000}"/>
@@ -5547,7 +5598,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5571,6 +5622,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000003000000}"/>
@@ -5580,7 +5632,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5604,6 +5656,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000004000000}"/>
@@ -5613,7 +5666,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5637,6 +5690,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000005000000}"/>
@@ -5646,7 +5700,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5670,6 +5724,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000006000000}"/>
@@ -5679,7 +5734,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5703,6 +5758,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000007000000}"/>
@@ -5712,7 +5768,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5736,6 +5792,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000008000000}"/>
@@ -5745,7 +5802,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5769,6 +5826,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-000009000000}"/>
@@ -5778,7 +5836,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5802,6 +5860,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-00000A000000}"/>
@@ -5811,7 +5870,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5835,6 +5894,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0400-00000B000000}"/>
@@ -5844,7 +5904,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5873,6 +5933,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000002000000}"/>
@@ -5882,7 +5943,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5906,6 +5967,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000003000000}"/>
@@ -5915,7 +5977,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5939,6 +6001,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000004000000}"/>
@@ -5948,7 +6011,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -5972,6 +6035,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000005000000}"/>
@@ -5981,7 +6045,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6005,6 +6069,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000006000000}"/>
@@ -6014,7 +6079,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6038,6 +6103,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000007000000}"/>
@@ -6047,7 +6113,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6071,6 +6137,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000008000000}"/>
@@ -6080,7 +6147,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6104,6 +6171,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000009000000}"/>
@@ -6113,7 +6181,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6137,6 +6205,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-00000A000000}"/>
@@ -6146,7 +6215,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6170,6 +6239,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-00000B000000}"/>
@@ -6179,7 +6249,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6301,9 +6371,389 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000008000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000A000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId16"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000B000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Image 11" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Image 12" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId20"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000D000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Image 13" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000E000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1600200" cy="361950"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6327,49 +6777,17 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 5" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000006000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1600200" cy="361950"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+        <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000007000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000004000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6399,43 +6817,11 @@
     <xdr:ext cx="1600200" cy="361950"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+        <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000008000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Image 8" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-000009000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000005000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6459,49 +6845,17 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1600200" cy="361950"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+        <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000A000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="11" name="Image 10" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000B000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6525,49 +6879,17 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1600200" cy="361950"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Image 11" descr="Picture">
+        <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000C000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Image 12" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000D000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000007000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -6591,242 +6913,6 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Image 13" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0600-00000E000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 2" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000003000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Image 3" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000004000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image 4" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000005000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Image 5" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000006000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1600200" cy="361950"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Image 6" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000007000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
@@ -6834,6 +6920,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000008000000}"/>
@@ -6843,7 +6930,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6867,6 +6954,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-000009000000}"/>
@@ -6876,7 +6964,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6900,6 +6988,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-00000A000000}"/>
@@ -6909,7 +6998,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6933,6 +7022,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0700-00000B000000}"/>
@@ -6942,7 +7032,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -6971,6 +7061,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Image 1" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000002000000}"/>
@@ -6980,7 +7071,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -7004,6 +7095,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="3" name="Image 2" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000003000000}"/>
@@ -7013,7 +7105,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -7037,6 +7129,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="4" name="Image 3" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000004000000}"/>
@@ -7046,7 +7139,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -7070,6 +7163,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="Image 4" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000005000000}"/>
@@ -7079,7 +7173,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -7103,6 +7197,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="6" name="Image 5" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000006000000}"/>
@@ -7112,7 +7207,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -7136,6 +7231,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="7" name="Image 6" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000007000000}"/>
@@ -7145,7 +7241,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -7169,6 +7265,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="8" name="Image 7" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000008000000}"/>
@@ -7178,7 +7275,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -7202,6 +7299,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="9" name="Image 8" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-000009000000}"/>
@@ -7211,7 +7309,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -7235,6 +7333,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="10" name="Image 9" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-00000A000000}"/>
@@ -7244,7 +7343,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -7268,6 +7367,7 @@
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="11" name="Image 10" descr="Picture">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0800-00000B000000}"/>
@@ -7277,7 +7377,7 @@
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>

</xml_diff>